<commit_message>
update C0004 AC scan data and BTMS model
</commit_message>
<xml_diff>
--- a/data/C0004/C0004R02_PARK25_AC_1D_SCAN.xlsx
+++ b/data/C0004/C0004R02_PARK25_AC_1D_SCAN.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Parameter scan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Parameter scan'!$A$1:$R$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$S$151</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R151"/>
+  <dimension ref="A1:S151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -468,6 +468,7 @@
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="19" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -561,6 +562,11 @@
           <t>dTmax_landing_C</t>
         </is>
       </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>m_bottom_plate_kg</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -619,6 +625,9 @@
       <c r="R2" s="4" t="n">
         <v>0.5368954238008357</v>
       </c>
+      <c r="S2" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -677,6 +686,9 @@
       <c r="R3" s="4" t="n">
         <v>0.5334646077005232</v>
       </c>
+      <c r="S3" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -735,6 +747,9 @@
       <c r="R4" s="4" t="n">
         <v>0.5301693847967002</v>
       </c>
+      <c r="S4" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -793,6 +808,9 @@
       <c r="R5" s="4" t="n">
         <v>0.5270045860690189</v>
       </c>
+      <c r="S5" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -851,6 +869,9 @@
       <c r="R6" s="4" t="n">
         <v>0.5239649067264551</v>
       </c>
+      <c r="S6" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -909,6 +930,9 @@
       <c r="R7" s="4" t="n">
         <v>0.5380717592994131</v>
       </c>
+      <c r="S7" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -967,6 +991,9 @@
       <c r="R8" s="4" t="n">
         <v>0.5346525678616061</v>
       </c>
+      <c r="S8" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1025,6 +1052,9 @@
       <c r="R9" s="4" t="n">
         <v>0.5313663298553877</v>
       </c>
+      <c r="S9" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -1083,6 +1113,9 @@
       <c r="R10" s="4" t="n">
         <v>0.5282081770867819</v>
       </c>
+      <c r="S10" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1141,6 +1174,9 @@
       <c r="R11" s="4" t="n">
         <v>0.5251730798889938</v>
       </c>
+      <c r="S11" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1199,6 +1235,9 @@
       <c r="R12" s="4" t="n">
         <v>0.5392218144075542</v>
       </c>
+      <c r="S12" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1257,6 +1296,9 @@
       <c r="R13" s="4" t="n">
         <v>0.5358147357274348</v>
       </c>
+      <c r="S13" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1315,6 +1357,9 @@
       <c r="R14" s="4" t="n">
         <v>0.5325380043194414</v>
       </c>
+      <c r="S14" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1373,6 +1418,9 @@
       <c r="R15" s="4" t="n">
         <v>0.5293870408876415</v>
       </c>
+      <c r="S15" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1431,6 +1479,9 @@
       <c r="R16" s="4" t="n">
         <v>0.5263570815276495</v>
       </c>
+      <c r="S16" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1489,6 +1540,9 @@
       <c r="R17" s="4" t="n">
         <v>0.5403463008839822</v>
       </c>
+      <c r="S17" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1547,6 +1601,9 @@
       <c r="R18" s="4" t="n">
         <v>0.5369517815769029</v>
       </c>
+      <c r="S18" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1605,6 +1662,9 @@
       <c r="R19" s="4" t="n">
         <v>0.5336850392380441</v>
       </c>
+      <c r="S19" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1663,6 +1723,9 @@
       <c r="R20" s="4" t="n">
         <v>0.5305417715969796</v>
       </c>
+      <c r="S20" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1721,6 +1784,9 @@
       <c r="R21" s="4" t="n">
         <v>0.5275174711295918</v>
       </c>
+      <c r="S21" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1779,6 +1845,9 @@
       <c r="R22" s="4" t="n">
         <v>0.5414459094455779</v>
       </c>
+      <c r="S22" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1837,6 +1906,9 @@
       <c r="R23" s="4" t="n">
         <v>0.53806435683655</v>
       </c>
+      <c r="S23" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1895,6 +1967,9 @@
       <c r="R24" s="4" t="n">
         <v>0.5348080487574833</v>
       </c>
+      <c r="S24" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1953,6 +2028,9 @@
       <c r="R25" s="4" t="n">
         <v>0.5316729481746663</v>
       </c>
+      <c r="S25" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -2011,6 +2089,9 @@
       <c r="R26" s="4" t="n">
         <v>0.5286547945673306</v>
       </c>
+      <c r="S26" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -2069,6 +2150,9 @@
       <c r="R27" s="4" t="n">
         <v>0.5198907877640551</v>
       </c>
+      <c r="S27" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -2127,6 +2211,9 @@
       <c r="R28" s="4" t="n">
         <v>0.5172161798949375</v>
       </c>
+      <c r="S28" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -2185,6 +2272,9 @@
       <c r="R29" s="4" t="n">
         <v>0.5147055665934488</v>
       </c>
+      <c r="S29" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -2243,6 +2333,9 @@
       <c r="R30" s="4" t="n">
         <v>0.5123450222473238</v>
       </c>
+      <c r="S30" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -2301,6 +2394,9 @@
       <c r="R31" s="4" t="n">
         <v>0.5101220508098265</v>
       </c>
+      <c r="S31" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -2359,6 +2455,9 @@
       <c r="R32" s="4" t="n">
         <v>0.5209159319710821</v>
       </c>
+      <c r="S32" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -2417,6 +2516,9 @@
       <c r="R33" s="4" t="n">
         <v>0.5182383224105109</v>
       </c>
+      <c r="S33" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -2475,6 +2577,9 @@
       <c r="R34" s="4" t="n">
         <v>0.5157240733798503</v>
       </c>
+      <c r="S34" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -2533,6 +2638,9 @@
       <c r="R35" s="4" t="n">
         <v>0.5133593991112662</v>
       </c>
+      <c r="S35" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -2591,6 +2699,9 @@
       <c r="R36" s="4" t="n">
         <v>0.5111319170750406</v>
       </c>
+      <c r="S36" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2649,6 +2760,9 @@
       <c r="R37" s="4" t="n">
         <v>0.521920643439465</v>
       </c>
+      <c r="S37" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2707,6 +2821,9 @@
       <c r="R38" s="4" t="n">
         <v>0.5192403137990311</v>
       </c>
+      <c r="S38" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2765,6 +2882,9 @@
       <c r="R39" s="4" t="n">
         <v>0.516722701407538</v>
       </c>
+      <c r="S39" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -2823,6 +2943,9 @@
       <c r="R40" s="4" t="n">
         <v>0.5143541596690469</v>
       </c>
+      <c r="S40" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -2881,6 +3004,9 @@
       <c r="R41" s="4" t="n">
         <v>0.5121224192565563</v>
       </c>
+      <c r="S41" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -2939,6 +3065,9 @@
       <c r="R42" s="4" t="n">
         <v>0.5229055312514816</v>
       </c>
+      <c r="S42" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2997,6 +3126,9 @@
       <c r="R43" s="4" t="n">
         <v>0.5202227502316177</v>
       </c>
+      <c r="S43" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -3055,6 +3187,9 @@
       <c r="R44" s="4" t="n">
         <v>0.5177020348113928</v>
       </c>
+      <c r="S44" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -3113,6 +3248,9 @@
       <c r="R45" s="4" t="n">
         <v>0.5153298768322259</v>
       </c>
+      <c r="S45" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -3171,6 +3309,9 @@
       <c r="R46" s="4" t="n">
         <v>0.5130941197941468</v>
       </c>
+      <c r="S46" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -3229,6 +3370,9 @@
       <c r="R47" s="4" t="n">
         <v>0.5238711767614248</v>
       </c>
+      <c r="S47" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
@@ -3287,6 +3431,9 @@
       <c r="R48" s="4" t="n">
         <v>0.5211862007987875</v>
       </c>
+      <c r="S48" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -3345,6 +3492,9 @@
       <c r="R49" s="4" t="n">
         <v>0.5186626312381577</v>
       </c>
+      <c r="S49" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -3403,6 +3553,9 @@
       <c r="R50" s="4" t="n">
         <v>0.5162870975674494</v>
       </c>
+      <c r="S50" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -3461,6 +3614,9 @@
       <c r="R51" s="4" t="n">
         <v>0.5140475556821684</v>
       </c>
+      <c r="S51" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
@@ -3519,6 +3675,9 @@
       <c r="R52" s="4" t="n">
         <v>0.504097491548599</v>
       </c>
+      <c r="S52" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
@@ -3577,6 +3736,9 @@
       <c r="R53" s="4" t="n">
         <v>0.5012753935234144</v>
       </c>
+      <c r="S53" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
@@ -3635,6 +3797,9 @@
       <c r="R54" s="4" t="n">
         <v>0.4986316679152409</v>
       </c>
+      <c r="S54" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -3693,6 +3858,9 @@
       <c r="R55" s="4" t="n">
         <v>0.4961506315406012</v>
       </c>
+      <c r="S55" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -3751,6 +3919,9 @@
       <c r="R56" s="4" t="n">
         <v>0.4938182818742831</v>
       </c>
+      <c r="S56" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -3809,6 +3980,9 @@
       <c r="R57" s="4" t="n">
         <v>0.5052030685097009</v>
       </c>
+      <c r="S57" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -3867,6 +4041,9 @@
       <c r="R58" s="4" t="n">
         <v>0.5023766949468396</v>
       </c>
+      <c r="S58" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -3925,6 +4102,9 @@
       <c r="R59" s="4" t="n">
         <v>0.4997281199767869</v>
       </c>
+      <c r="S59" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
@@ -3983,6 +4163,9 @@
       <c r="R60" s="4" t="n">
         <v>0.4972418014631401</v>
       </c>
+      <c r="S60" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -4041,6 +4224,9 @@
       <c r="R61" s="4" t="n">
         <v>0.4949038500073542</v>
       </c>
+      <c r="S61" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -4099,6 +4285,9 @@
       <c r="R62" s="4" t="n">
         <v>0.5062867448578103</v>
       </c>
+      <c r="S62" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -4157,6 +4346,9 @@
       <c r="R63" s="4" t="n">
         <v>0.503456411509525</v>
       </c>
+      <c r="S63" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
@@ -4215,6 +4407,9 @@
       <c r="R64" s="4" t="n">
         <v>0.5008032906264361</v>
       </c>
+      <c r="S64" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -4273,6 +4468,9 @@
       <c r="R65" s="4" t="n">
         <v>0.4983119807252905</v>
       </c>
+      <c r="S65" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
@@ -4331,6 +4529,9 @@
       <c r="R66" s="4" t="n">
         <v>0.4959687054881385</v>
       </c>
+      <c r="S66" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -4389,6 +4590,9 @@
       <c r="R67" s="4" t="n">
         <v>0.5073491703974327</v>
       </c>
+      <c r="S67" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
@@ -4447,6 +4651,9 @@
       <c r="R68" s="4" t="n">
         <v>0.5045151786946533</v>
       </c>
+      <c r="S68" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -4505,6 +4712,9 @@
       <c r="R69" s="4" t="n">
         <v>0.5018578020829665</v>
       </c>
+      <c r="S69" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
@@ -4563,6 +4773,9 @@
       <c r="R70" s="4" t="n">
         <v>0.4993617792480123</v>
       </c>
+      <c r="S70" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
@@ -4621,6 +4834,9 @@
       <c r="R71" s="4" t="n">
         <v>0.4970134468215761</v>
       </c>
+      <c r="S71" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
@@ -4679,6 +4895,9 @@
       <c r="R72" s="4" t="n">
         <v>0.5083909656832191</v>
       </c>
+      <c r="S72" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
@@ -4737,6 +4956,9 @@
       <c r="R73" s="4" t="n">
         <v>0.5055536034362689</v>
       </c>
+      <c r="S73" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
@@ -4795,6 +5017,9 @@
       <c r="R74" s="4" t="n">
         <v>0.5028922486531116</v>
       </c>
+      <c r="S74" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
@@ -4853,6 +5078,9 @@
       <c r="R75" s="4" t="n">
         <v>0.5003917796212676</v>
       </c>
+      <c r="S75" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
@@ -4911,6 +5139,9 @@
       <c r="R76" s="4" t="n">
         <v>0.498038645713244</v>
       </c>
+      <c r="S76" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
@@ -4969,6 +5200,9 @@
       <c r="R77" s="4" t="n">
         <v>0.4899918843462459</v>
       </c>
+      <c r="S77" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -5027,6 +5261,9 @@
       <c r="R78" s="4" t="n">
         <v>0.4870438649504365</v>
       </c>
+      <c r="S78" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -5085,6 +5322,9 @@
       <c r="R79" s="4" t="n">
         <v>0.48428700165897</v>
       </c>
+      <c r="S79" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
@@ -5143,6 +5383,9 @@
       <c r="R80" s="4" t="n">
         <v>0.4817039923981596</v>
       </c>
+      <c r="S80" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
@@ -5201,6 +5444,9 @@
       <c r="R81" s="4" t="n">
         <v>0.4792794551700723</v>
       </c>
+      <c r="S81" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
@@ -5259,6 +5505,9 @@
       <c r="R82" s="4" t="n">
         <v>0.491170677129908</v>
       </c>
+      <c r="S82" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -5317,6 +5566,9 @@
       <c r="R83" s="4" t="n">
         <v>0.4882171004965699</v>
       </c>
+      <c r="S83" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
@@ -5375,6 +5627,9 @@
       <c r="R84" s="4" t="n">
         <v>0.4854541706179134</v>
       </c>
+      <c r="S84" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
@@ -5433,6 +5688,9 @@
       <c r="R85" s="4" t="n">
         <v>0.48286472709691</v>
       </c>
+      <c r="S85" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
@@ -5491,6 +5749,9 @@
       <c r="R86" s="4" t="n">
         <v>0.4804335000724862</v>
       </c>
+      <c r="S86" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
@@ -5549,6 +5810,9 @@
       <c r="R87" s="4" t="n">
         <v>0.4923262571677967</v>
       </c>
+      <c r="S87" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
@@ -5607,6 +5871,9 @@
       <c r="R88" s="4" t="n">
         <v>0.4893674777267663</v>
       </c>
+      <c r="S88" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
@@ -5665,6 +5932,9 @@
       <c r="R89" s="4" t="n">
         <v>0.4865988194156543</v>
       </c>
+      <c r="S89" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
@@ -5723,6 +5993,9 @@
       <c r="R90" s="4" t="n">
         <v>0.4840032635932943</v>
       </c>
+      <c r="S90" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
@@ -5781,6 +6054,9 @@
       <c r="R91" s="4" t="n">
         <v>0.4815656529070651</v>
       </c>
+      <c r="S91" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
@@ -5839,6 +6115,9 @@
       <c r="R92" s="4" t="n">
         <v>0.493459305353845</v>
       </c>
+      <c r="S92" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
@@ -5897,6 +6176,9 @@
       <c r="R93" s="4" t="n">
         <v>0.4904956619517122</v>
       </c>
+      <c r="S93" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
@@ -5955,6 +6237,9 @@
       <c r="R94" s="4" t="n">
         <v>0.487721599016858</v>
       </c>
+      <c r="S94" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
@@ -6013,6 +6298,9 @@
       <c r="R95" s="4" t="n">
         <v>0.4851202396219136</v>
       </c>
+      <c r="S95" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
@@ -6071,6 +6359,9 @@
       <c r="R96" s="4" t="n">
         <v>0.4826765391846024</v>
       </c>
+      <c r="S96" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
@@ -6129,6 +6420,9 @@
       <c r="R97" s="4" t="n">
         <v>0.4945704724028772</v>
       </c>
+      <c r="S97" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
@@ -6187,6 +6481,9 @@
       <c r="R98" s="4" t="n">
         <v>0.4916022890346667</v>
       </c>
+      <c r="S98" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
@@ -6245,6 +6542,9 @@
       <c r="R99" s="4" t="n">
         <v>0.4888231316008955</v>
       </c>
+      <c r="S99" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -6303,6 +6603,9 @@
       <c r="R100" s="4" t="n">
         <v>0.4862162647333719</v>
       </c>
+      <c r="S100" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -6361,6 +6664,9 @@
       <c r="R101" s="4" t="n">
         <v>0.4837667567801276</v>
       </c>
+      <c r="S101" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
@@ -6419,6 +6725,9 @@
       <c r="R102" s="4" t="n">
         <v>0.4771060681293235</v>
       </c>
+      <c r="S102" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -6477,6 +6786,9 @@
       <c r="R103" s="4" t="n">
         <v>0.4740501176885061</v>
       </c>
+      <c r="S103" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
@@ -6535,6 +6847,9 @@
       <c r="R104" s="4" t="n">
         <v>0.4711968305755505</v>
       </c>
+      <c r="S104" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
@@ -6593,6 +6908,9 @@
       <c r="R105" s="4" t="n">
         <v>0.4685273856120205</v>
       </c>
+      <c r="S105" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
@@ -6651,6 +6969,9 @@
       <c r="R106" s="4" t="n">
         <v>0.4660251161521529</v>
       </c>
+      <c r="S106" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
@@ -6709,6 +7030,9 @@
       <c r="R107" s="4" t="n">
         <v>0.4783521579826981</v>
       </c>
+      <c r="S107" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
@@ -6767,6 +7091,9 @@
       <c r="R108" s="4" t="n">
         <v>0.4752892895199636</v>
       </c>
+      <c r="S108" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -6825,6 +7152,9 @@
       <c r="R109" s="4" t="n">
         <v>0.4724286556226005</v>
       </c>
+      <c r="S109" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
@@ -6883,6 +7213,9 @@
       <c r="R110" s="4" t="n">
         <v>0.4697515745012666</v>
       </c>
+      <c r="S110" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -6941,6 +7274,9 @@
       <c r="R111" s="4" t="n">
         <v>0.4672414882579687</v>
       </c>
+      <c r="S111" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
@@ -6999,6 +7335,9 @@
       <c r="R112" s="4" t="n">
         <v>0.4795739067410238</v>
       </c>
+      <c r="S112" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
@@ -7057,6 +7396,9 @@
       <c r="R113" s="4" t="n">
         <v>0.476504513502654</v>
       </c>
+      <c r="S113" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
@@ -7115,6 +7457,9 @@
       <c r="R114" s="4" t="n">
         <v>0.4736369054216993</v>
       </c>
+      <c r="S114" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -7173,6 +7518,9 @@
       <c r="R115" s="4" t="n">
         <v>0.4709525407704973</v>
       </c>
+      <c r="S115" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
@@ -7231,6 +7579,9 @@
       <c r="R116" s="4" t="n">
         <v>0.4684349712753075</v>
       </c>
+      <c r="S116" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
@@ -7289,6 +7640,9 @@
       <c r="R117" s="4" t="n">
         <v>0.4807720172864052</v>
       </c>
+      <c r="S117" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
@@ -7347,6 +7701,9 @@
       <c r="R118" s="4" t="n">
         <v>0.4776964759481501</v>
       </c>
+      <c r="S118" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
@@ -7405,6 +7762,9 @@
       <c r="R119" s="4" t="n">
         <v>0.4748222511066587</v>
       </c>
+      <c r="S119" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
@@ -7463,6 +7823,9 @@
       <c r="R120" s="4" t="n">
         <v>0.4721309416184383</v>
       </c>
+      <c r="S120" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
@@ -7521,6 +7884,9 @@
       <c r="R121" s="4" t="n">
         <v>0.469606209578167</v>
       </c>
+      <c r="S121" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
@@ -7579,6 +7945,9 @@
       <c r="R122" s="4" t="n">
         <v>0.4819471618444808</v>
       </c>
+      <c r="S122" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -7637,6 +8006,9 @@
       <c r="R123" s="4" t="n">
         <v>0.4788658332550852</v>
       </c>
+      <c r="S123" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
@@ -7695,6 +8067,9 @@
       <c r="R124" s="4" t="n">
         <v>0.4759853345686977</v>
       </c>
+      <c r="S124" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -7753,6 +8128,9 @@
       <c r="R125" s="4" t="n">
         <v>0.473287405608346</v>
       </c>
+      <c r="S125" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
@@ -7811,6 +8189,9 @@
       <c r="R126" s="4" t="n">
         <v>0.4707558194571462</v>
       </c>
+      <c r="S126" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -7869,6 +8250,9 @@
       <c r="R127" s="4" t="n">
         <v>0.4651566620784138</v>
       </c>
+      <c r="S127" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
@@ -7927,6 +8311,9 @@
       <c r="R128" s="4" t="n">
         <v>0.4620087866060629</v>
       </c>
+      <c r="S128" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
@@ -7985,6 +8372,9 @@
       <c r="R129" s="4" t="n">
         <v>0.4590739030683153</v>
       </c>
+      <c r="S129" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
@@ -8043,6 +8433,9 @@
       <c r="R130" s="4" t="n">
         <v>0.4563317695708662</v>
       </c>
+      <c r="S130" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -8101,6 +8494,9 @@
       <c r="R131" s="4" t="n">
         <v>0.4537645271155739</v>
       </c>
+      <c r="S131" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
@@ -8159,6 +8555,9 @@
       <c r="R132" s="4" t="n">
         <v>0.4664645120159747</v>
       </c>
+      <c r="S132" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
@@ -8217,6 +8616,9 @@
       <c r="R133" s="4" t="n">
         <v>0.4633082896256084</v>
       </c>
+      <c r="S133" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
@@ -8275,6 +8677,9 @@
       <c r="R134" s="4" t="n">
         <v>0.4603647277500755</v>
       </c>
+      <c r="S134" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
@@ -8333,6 +8738,9 @@
       <c r="R135" s="4" t="n">
         <v>0.457613718215427</v>
       </c>
+      <c r="S135" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
@@ -8391,6 +8799,9 @@
       <c r="R136" s="4" t="n">
         <v>0.4550375046915462</v>
       </c>
+      <c r="S136" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
@@ -8449,6 +8860,9 @@
       <c r="R137" s="4" t="n">
         <v>0.4677470772235495</v>
       </c>
+      <c r="S137" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
@@ -8507,6 +8921,9 @@
       <c r="R138" s="4" t="n">
         <v>0.464582937442394</v>
       </c>
+      <c r="S138" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
@@ -8565,6 +8982,9 @@
       <c r="R139" s="4" t="n">
         <v>0.4616311017344046</v>
       </c>
+      <c r="S139" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
@@ -8623,6 +9043,9 @@
       <c r="R140" s="4" t="n">
         <v>0.458871596962183</v>
       </c>
+      <c r="S140" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
@@ -8681,6 +9104,9 @@
       <c r="R141" s="4" t="n">
         <v>0.4562867708762539</v>
       </c>
+      <c r="S141" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
@@ -8739,6 +9165,9 @@
       <c r="R142" s="4" t="n">
         <v>0.4690050748767618</v>
       </c>
+      <c r="S142" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -8797,6 +9226,9 @@
       <c r="R143" s="4" t="n">
         <v>0.4658334299621245</v>
       </c>
+      <c r="S143" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
@@ -8855,6 +9287,9 @@
       <c r="R144" s="4" t="n">
         <v>0.4628737091735289</v>
       </c>
+      <c r="S144" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
@@ -8913,6 +9348,9 @@
       <c r="R145" s="4" t="n">
         <v>0.4601060755517565</v>
       </c>
+      <c r="S145" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
@@ -8971,6 +9409,9 @@
       <c r="R146" s="4" t="n">
         <v>0.4575129821893498</v>
       </c>
+      <c r="S146" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
@@ -9029,6 +9470,9 @@
       <c r="R147" s="4" t="n">
         <v>0.4702391913435733</v>
       </c>
+      <c r="S147" s="4" t="n">
+        <v>0.6201198</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
@@ -9087,6 +9531,9 @@
       <c r="R148" s="4" t="n">
         <v>0.4670604370240881</v>
       </c>
+      <c r="S148" s="4" t="n">
+        <v>0.6834456</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
@@ -9145,6 +9592,9 @@
       <c r="R149" s="4" t="n">
         <v>0.4640932048196902</v>
       </c>
+      <c r="S149" s="4" t="n">
+        <v>0.7498494</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
@@ -9203,6 +9653,9 @@
       <c r="R150" s="4" t="n">
         <v>0.4613177949270337</v>
       </c>
+      <c r="S150" s="4" t="n">
+        <v>0.8193312</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
@@ -9261,9 +9714,12 @@
       <c r="R151" s="4" t="n">
         <v>0.458716766899272</v>
       </c>
+      <c r="S151" s="4" t="n">
+        <v>0.8918910000000001</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R151"/>
+  <autoFilter ref="A1:S151"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>